<commit_message>
Add GPIO TestPlan Excel generated from extracted testcases (TestRepo/gpio on main)
</commit_message>
<xml_diff>
--- a/Test_Output/GPIO/GPIO_TestPlan.xlsx
+++ b/Test_Output/GPIO/GPIO_TestPlan.xlsx
@@ -7,8 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="GPIO_TestPlan" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="TestPlan" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -64,14 +63,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -440,19 +438,19 @@
   <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="53" customWidth="1" min="3" max="3"/>
-    <col width="35" customWidth="1" min="4" max="4"/>
-    <col width="80" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="57" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
-    <col width="36" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="36" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="23" customWidth="1" min="3" max="3"/>
+    <col width="33" customWidth="1" min="4" max="4"/>
+    <col width="66" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="34" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="34" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -535,7 +533,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>GPIO register write/read test</t>
+          <t>gpio_reg_wr_rd</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -545,7 +543,7 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>Validate GPIO register write and read back consistency.</t>
+          <t>Validate GPIO register write and read behavior.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -565,11 +563,7 @@
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>1. Initialize the GPIO module.
-2. Write known values to GPIO-related registers.
-3. Read back the written registers.
-4. Compare read values with the written values.
-5. Log pass/fail status.</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -602,7 +596,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Negative-edge interrupt with alternate pads enabled</t>
+          <t>nedge_alternate_pads_en</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -612,7 +606,7 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Verify GPIO negative-edge interrupt behavior when alternate pads are enabled.</t>
+          <t>Verify GPIO negative-edge behavior on alternate pads when enabled.</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -632,11 +626,7 @@
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>1. Initialize the GPIO module.
-2. Enable negative-edge interrupt on alternate pads.
-3. Stimulate negative-edge transitions on enabled pads.
-4. Monitor and record interrupt events.
-5. Report results.</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -669,7 +659,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Negative-edge interrupt enable</t>
+          <t>negedge_intr_en</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -679,7 +669,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Check that enabling negative-edge interrupts triggers events on falling edges.</t>
+          <t>Verify GPIO negative-edge interrupt enable functionality.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -699,11 +689,7 @@
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>1. Initialize the GPIO module.
-2. Configure negative-edge interrupt on selected pads.
-3. Apply falling-edge signals to the pads.
-4. Observe interrupt signaling and capture status.
-5. Summarize pass/fail.</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -736,7 +722,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Positive-edge interrupt with all pads enabled</t>
+          <t>pedge_all_pads_en</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -746,7 +732,7 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Validate GPIO positive-edge interrupts when enabled on all pads.</t>
+          <t>Verify GPIO positive-edge behavior with all pads enabled.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -766,11 +752,7 @@
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>1. Initialize the GPIO module.
-2. Enable positive-edge interrupt on all pads.
-3. Generate rising edges on multiple pads.
-4. Observe interrupt activity and log events.
-5. Determine overall result.</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -803,7 +785,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Positive-edge interrupt with alternate pads enabled</t>
+          <t>pedge_alternate_pads_en</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -813,7 +795,7 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Verify positive-edge interrupt functionality when alternate pads are enabled.</t>
+          <t>Verify GPIO positive-edge behavior on alternate pads when enabled.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -833,11 +815,7 @@
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>1. Initialize the GPIO module.
-2. Enable positive-edge interrupt on alternate pads.
-3. Apply rising-edge signals to enabled pads.
-4. Monitor interrupt occurrences and capture status.
-5. Conclude pass/fail.</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -865,115 +843,4 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>TestPlan Generation Summary</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>Generated At (IST)</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-06-17 13:42:32 IST</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>IP_NAME</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>GPIO</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Source Scope</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>TestRepo/gpio</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>Output File</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Test_Output/GPIO/GPIO_TestPlan.xlsx</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>Source Folders</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>https://github.com/titusbspgit/SemiTestSuite/tree/main/TestRepo/gpio/gpio_reg_wr_rd_test</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>https://github.com/titusbspgit/SemiTestSuite/tree/main/TestRepo/gpio/test_gpio_nedge_alternate_pads_en</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>https://github.com/titusbspgit/SemiTestSuite/tree/main/TestRepo/gpio/test_gpio_negedge_intr_en</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>https://github.com/titusbspgit/SemiTestSuite/tree/main/TestRepo/gpio/test_gpio_pedge_all_pads_en</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>https://github.com/titusbspgit/SemiTestSuite/tree/main/TestRepo/gpio/test_gpio_pedge_alternate_pads_en</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>